<commit_message>
Ajusta formato dos Contatos na importação de Clientes
Troca "Nome;E-mail;Telefone" por blocos '{ID, Nome, E-mail, Telefone,
Setor}' separados por ';', igual ao formato que a Ingrid já usa.

O ID vira contact.identifier e passa a ser a chave preferida pra achar
um contato já existente numa reimportação (mais estável que e-mail/
telefone, que podem mudar). O Setor não tem coluna própria no Contact,
então vai pro additional_attributes (jsonb) como "setor".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/clientes-modelo.xlsx
+++ b/public/downloads/clientes-modelo.xlsx
@@ -416,7 +416,7 @@
         <v>IM</v>
       </c>
       <c r="F1" t="str">
-        <v>Contatos (Separado por '{}')</v>
+        <v>Contatos (formato: {ID, Nome, E-mail, Telefone, Setor})</v>
       </c>
       <c r="G1" t="str">
         <v>Rua</v>
@@ -460,7 +460,7 @@
         <v>987654</v>
       </c>
       <c r="F2" t="str">
-        <v>Maria Silva;maria.silva@empresaexemplo.com.br;+5511999999999{}João Souza;joao.souza@empresaexemplo.com.br;+5511988888888</v>
+        <v>{1294494, Maria Silva, maria.silva@empresaexemplo.com.br, 5511999999999, Comercial};{1294495, João Souza, joao.souza@empresaexemplo.com.br, 5511988888888, Financeiro}</v>
       </c>
       <c r="G2" t="str">
         <v>Rua das Flores</v>
@@ -504,7 +504,7 @@
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>Ana Pereira;ana.pereira@gmail.com;+5511977777777</v>
+        <v>{1294496, Ana Pereira, ana.pereira@gmail.com, 5511977777777, Diretoria}</v>
       </c>
       <c r="G3" t="str">
         <v>Av. Paulista</v>

</xml_diff>